<commit_message>
feat: indosbert vector embedding
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14">
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>9</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="20">
@@ -1089,7 +1089,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25">
@@ -1145,7 +1145,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30">
@@ -1313,7 +1313,7 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
@@ -1341,7 +1341,7 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34">
@@ -1369,7 +1369,7 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="35">
@@ -1509,7 +1509,7 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>9</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="40">
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41">
@@ -1649,7 +1649,7 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="45">
@@ -1677,7 +1677,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="46">
@@ -1705,7 +1705,7 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="47">
@@ -1845,7 +1845,7 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="52">
@@ -1901,7 +1901,7 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="54">
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="56">
@@ -2013,7 +2013,7 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="58">
@@ -2097,7 +2097,7 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="61">
@@ -2125,7 +2125,7 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="62">
@@ -2153,7 +2153,7 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="63">
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="71">
@@ -2433,7 +2433,7 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="73">
@@ -2545,7 +2545,7 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>-1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="77">
@@ -2741,7 +2741,7 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="84">
@@ -2797,7 +2797,7 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="86">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="89">
@@ -3133,7 +3133,7 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="98">
@@ -3217,7 +3217,7 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="101">
@@ -3273,7 +3273,7 @@
         </is>
       </c>
       <c r="F102" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="103">
@@ -3357,7 +3357,7 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="106">
@@ -3413,7 +3413,7 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>11</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="108">
@@ -3441,7 +3441,7 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="109">
@@ -3497,7 +3497,7 @@
         </is>
       </c>
       <c r="F110" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="111">
@@ -3525,7 +3525,7 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="112">
@@ -3581,7 +3581,7 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="114">
@@ -3637,7 +3637,7 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="116">
@@ -3693,7 +3693,7 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="118">
@@ -3861,7 +3861,7 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="124">
@@ -4225,7 +4225,7 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="137">
@@ -4253,7 +4253,7 @@
         </is>
       </c>
       <c r="F137" t="n">
-        <v>-1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="138">
@@ -4785,7 +4785,7 @@
         </is>
       </c>
       <c r="F156" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="157">
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="F166" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="167">
@@ -5121,7 +5121,7 @@
         </is>
       </c>
       <c r="F168" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="169">
@@ -5205,7 +5205,7 @@
         </is>
       </c>
       <c r="F171" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="172">
@@ -5233,7 +5233,7 @@
         </is>
       </c>
       <c r="F172" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="173">
@@ -5317,7 +5317,7 @@
         </is>
       </c>
       <c r="F175" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="176">
@@ -5429,7 +5429,7 @@
         </is>
       </c>
       <c r="F179" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="180">
@@ -5597,7 +5597,7 @@
         </is>
       </c>
       <c r="F185" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="186">
@@ -5765,7 +5765,7 @@
         </is>
       </c>
       <c r="F191" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="192">
@@ -5905,7 +5905,7 @@
         </is>
       </c>
       <c r="F196" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="197">
@@ -6017,7 +6017,7 @@
         </is>
       </c>
       <c r="F200" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="201">
@@ -6129,7 +6129,7 @@
         </is>
       </c>
       <c r="F204" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="205">
@@ -6185,7 +6185,7 @@
         </is>
       </c>
       <c r="F206" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="207">
@@ -6269,7 +6269,7 @@
         </is>
       </c>
       <c r="F209" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="210">
@@ -6437,7 +6437,7 @@
         </is>
       </c>
       <c r="F215" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="216">
@@ -6577,7 +6577,7 @@
         </is>
       </c>
       <c r="F220" t="n">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="221">
@@ -6605,7 +6605,7 @@
         </is>
       </c>
       <c r="F221" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="222">
@@ -6661,7 +6661,7 @@
         </is>
       </c>
       <c r="F223" t="n">
-        <v>11</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="224">
@@ -7025,7 +7025,7 @@
         </is>
       </c>
       <c r="F236" t="n">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="237">
@@ -7137,7 +7137,7 @@
         </is>
       </c>
       <c r="F240" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="241">
@@ -7165,7 +7165,7 @@
         </is>
       </c>
       <c r="F241" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="242">
@@ -7333,7 +7333,7 @@
         </is>
       </c>
       <c r="F247" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="248">
@@ -7417,7 +7417,7 @@
         </is>
       </c>
       <c r="F250" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="251">
@@ -7837,7 +7837,7 @@
         </is>
       </c>
       <c r="F265" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="266">
@@ -7921,7 +7921,7 @@
         </is>
       </c>
       <c r="F268" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="269">
@@ -8061,7 +8061,7 @@
         </is>
       </c>
       <c r="F273" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="274">
@@ -8285,7 +8285,7 @@
         </is>
       </c>
       <c r="F281" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="282">
@@ -8565,7 +8565,7 @@
         </is>
       </c>
       <c r="F291" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="292">
@@ -8677,7 +8677,7 @@
         </is>
       </c>
       <c r="F295" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="296">
@@ -8761,7 +8761,7 @@
         </is>
       </c>
       <c r="F298" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="299">
@@ -8985,7 +8985,7 @@
         </is>
       </c>
       <c r="F306" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="307">
@@ -9069,7 +9069,7 @@
         </is>
       </c>
       <c r="F309" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="310">
@@ -9405,7 +9405,7 @@
         </is>
       </c>
       <c r="F321" t="n">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="322">
@@ -9601,7 +9601,7 @@
         </is>
       </c>
       <c r="F328" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="329">
@@ -9713,7 +9713,7 @@
         </is>
       </c>
       <c r="F332" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="333">
@@ -9797,7 +9797,7 @@
         </is>
       </c>
       <c r="F335" t="n">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="336">
@@ -9853,7 +9853,7 @@
         </is>
       </c>
       <c r="F337" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="338">
@@ -9909,7 +9909,7 @@
         </is>
       </c>
       <c r="F339" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="340">
@@ -9965,7 +9965,7 @@
         </is>
       </c>
       <c r="F341" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="342">
@@ -10077,7 +10077,7 @@
         </is>
       </c>
       <c r="F345" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="346">
@@ -10189,7 +10189,7 @@
         </is>
       </c>
       <c r="F349" t="n">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="350">
@@ -10217,7 +10217,7 @@
         </is>
       </c>
       <c r="F350" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="351">
@@ -10301,7 +10301,7 @@
         </is>
       </c>
       <c r="F353" t="n">
-        <v>-1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="354">
@@ -10357,7 +10357,7 @@
         </is>
       </c>
       <c r="F355" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="356">
@@ -10525,7 +10525,7 @@
         </is>
       </c>
       <c r="F361" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="362">
@@ -10693,7 +10693,7 @@
         </is>
       </c>
       <c r="F367" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="368">
@@ -10805,7 +10805,7 @@
         </is>
       </c>
       <c r="F371" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="372">
@@ -10861,7 +10861,7 @@
         </is>
       </c>
       <c r="F373" t="n">
-        <v>8</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="374">
@@ -10945,7 +10945,7 @@
         </is>
       </c>
       <c r="F376" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="377">
@@ -11001,7 +11001,7 @@
         </is>
       </c>
       <c r="F378" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="379">
@@ -11113,7 +11113,7 @@
         </is>
       </c>
       <c r="F382" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="383">
@@ -11141,7 +11141,7 @@
         </is>
       </c>
       <c r="F383" t="n">
-        <v>-1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="384">
@@ -11225,7 +11225,7 @@
         </is>
       </c>
       <c r="F386" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="387">
@@ -11253,7 +11253,7 @@
         </is>
       </c>
       <c r="F387" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="388">
@@ -11281,7 +11281,7 @@
         </is>
       </c>
       <c r="F388" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="389">
@@ -11393,7 +11393,7 @@
         </is>
       </c>
       <c r="F392" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="393">
@@ -11505,7 +11505,7 @@
         </is>
       </c>
       <c r="F396" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="397">
@@ -11645,7 +11645,7 @@
         </is>
       </c>
       <c r="F401" t="n">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="402">
@@ -11729,7 +11729,7 @@
         </is>
       </c>
       <c r="F404" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="405">
@@ -11897,7 +11897,7 @@
         </is>
       </c>
       <c r="F410" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="411">
@@ -11925,7 +11925,7 @@
         </is>
       </c>
       <c r="F411" t="n">
-        <v>11</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="412">
@@ -11953,7 +11953,7 @@
         </is>
       </c>
       <c r="F412" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="413">
@@ -12149,7 +12149,7 @@
         </is>
       </c>
       <c r="F419" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="420">
@@ -12345,7 +12345,7 @@
         </is>
       </c>
       <c r="F426" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="427">
@@ -12429,7 +12429,7 @@
         </is>
       </c>
       <c r="F429" t="n">
-        <v>-1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="430">
@@ -12457,7 +12457,7 @@
         </is>
       </c>
       <c r="F430" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="431">
@@ -12681,7 +12681,7 @@
         </is>
       </c>
       <c r="F438" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="439">
@@ -12709,7 +12709,7 @@
         </is>
       </c>
       <c r="F439" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="440">
@@ -12765,7 +12765,7 @@
         </is>
       </c>
       <c r="F441" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="442">
@@ -12793,7 +12793,7 @@
         </is>
       </c>
       <c r="F442" t="n">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="443">
@@ -12961,7 +12961,7 @@
         </is>
       </c>
       <c r="F448" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="449">
@@ -13045,7 +13045,7 @@
         </is>
       </c>
       <c r="F451" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="452">
@@ -13129,7 +13129,7 @@
         </is>
       </c>
       <c r="F454" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="455">
@@ -13241,7 +13241,7 @@
         </is>
       </c>
       <c r="F458" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="459">
@@ -13297,7 +13297,7 @@
         </is>
       </c>
       <c r="F460" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="461">
@@ -13437,7 +13437,7 @@
         </is>
       </c>
       <c r="F465" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="466">
@@ -13633,7 +13633,7 @@
         </is>
       </c>
       <c r="F472" t="n">
-        <v>8</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="473">
@@ -13773,7 +13773,7 @@
         </is>
       </c>
       <c r="F477" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="478">
@@ -13801,7 +13801,7 @@
         </is>
       </c>
       <c r="F478" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="479">
@@ -13913,7 +13913,7 @@
         </is>
       </c>
       <c r="F482" t="n">
-        <v>8</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="483">
@@ -14053,7 +14053,7 @@
         </is>
       </c>
       <c r="F487" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="488">
@@ -14081,7 +14081,7 @@
         </is>
       </c>
       <c r="F488" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="489">
@@ -14193,7 +14193,7 @@
         </is>
       </c>
       <c r="F492" t="n">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="493">
@@ -14417,7 +14417,7 @@
         </is>
       </c>
       <c r="F500" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="501">
@@ -14557,7 +14557,7 @@
         </is>
       </c>
       <c r="F505" t="n">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="506">
@@ -14781,7 +14781,7 @@
         </is>
       </c>
       <c r="F513" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="514">
@@ -14809,7 +14809,7 @@
         </is>
       </c>
       <c r="F514" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="515">
@@ -14977,7 +14977,7 @@
         </is>
       </c>
       <c r="F520" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="521">
@@ -15061,7 +15061,7 @@
         </is>
       </c>
       <c r="F523" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="524">
@@ -15117,7 +15117,7 @@
         </is>
       </c>
       <c r="F525" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="526">
@@ -15341,7 +15341,7 @@
         </is>
       </c>
       <c r="F533" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="534">
@@ -15453,7 +15453,7 @@
         </is>
       </c>
       <c r="F537" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="538">
@@ -15509,7 +15509,7 @@
         </is>
       </c>
       <c r="F539" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="540">
@@ -15565,7 +15565,7 @@
         </is>
       </c>
       <c r="F541" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="542">
@@ -15621,7 +15621,7 @@
         </is>
       </c>
       <c r="F543" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="544">
@@ -15873,7 +15873,7 @@
         </is>
       </c>
       <c r="F552" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="553">
@@ -16097,7 +16097,7 @@
         </is>
       </c>
       <c r="F560" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="561">
@@ -16125,7 +16125,7 @@
         </is>
       </c>
       <c r="F561" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="562">
@@ -16265,7 +16265,7 @@
         </is>
       </c>
       <c r="F566" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="567">
@@ -16293,7 +16293,7 @@
         </is>
       </c>
       <c r="F567" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="568">
@@ -16349,7 +16349,7 @@
         </is>
       </c>
       <c r="F569" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="570">
@@ -16489,7 +16489,7 @@
         </is>
       </c>
       <c r="F574" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="575">
@@ -16517,7 +16517,7 @@
         </is>
       </c>
       <c r="F575" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="576">
@@ -16545,7 +16545,7 @@
         </is>
       </c>
       <c r="F576" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="577">
@@ -16741,7 +16741,7 @@
         </is>
       </c>
       <c r="F583" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="584">
@@ -17077,7 +17077,7 @@
         </is>
       </c>
       <c r="F595" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="596">
@@ -17329,7 +17329,7 @@
         </is>
       </c>
       <c r="F604" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="605">
@@ -17469,7 +17469,7 @@
         </is>
       </c>
       <c r="F609" t="n">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="610">
@@ -17581,7 +17581,7 @@
         </is>
       </c>
       <c r="F613" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="614">
@@ -17609,7 +17609,7 @@
         </is>
       </c>
       <c r="F614" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="615">
@@ -17665,7 +17665,7 @@
         </is>
       </c>
       <c r="F616" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="617">
@@ -17693,7 +17693,7 @@
         </is>
       </c>
       <c r="F617" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="618">
@@ -17833,7 +17833,7 @@
         </is>
       </c>
       <c r="F622" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="623">
@@ -17917,7 +17917,7 @@
         </is>
       </c>
       <c r="F625" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="626">
@@ -18001,7 +18001,7 @@
         </is>
       </c>
       <c r="F628" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="629">
@@ -18057,7 +18057,7 @@
         </is>
       </c>
       <c r="F630" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="631">
@@ -18141,7 +18141,7 @@
         </is>
       </c>
       <c r="F633" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="634">
@@ -18169,7 +18169,7 @@
         </is>
       </c>
       <c r="F634" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="635">
@@ -18225,7 +18225,7 @@
         </is>
       </c>
       <c r="F636" t="n">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="637">
@@ -18449,7 +18449,7 @@
         </is>
       </c>
       <c r="F644" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="645">
@@ -18477,7 +18477,7 @@
         </is>
       </c>
       <c r="F645" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="646">
@@ -18505,7 +18505,7 @@
         </is>
       </c>
       <c r="F646" t="n">
-        <v>-1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="647">
@@ -18533,7 +18533,7 @@
         </is>
       </c>
       <c r="F647" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="648">
@@ -18589,7 +18589,7 @@
         </is>
       </c>
       <c r="F649" t="n">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="650">
@@ -18701,7 +18701,7 @@
         </is>
       </c>
       <c r="F653" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="654">
@@ -18841,7 +18841,7 @@
         </is>
       </c>
       <c r="F658" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="659">
@@ -19121,7 +19121,7 @@
         </is>
       </c>
       <c r="F668" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="669">
@@ -19149,7 +19149,7 @@
         </is>
       </c>
       <c r="F669" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="670">
@@ -19177,7 +19177,7 @@
         </is>
       </c>
       <c r="F670" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="671">
@@ -19289,7 +19289,7 @@
         </is>
       </c>
       <c r="F674" t="n">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="675">
@@ -19317,7 +19317,7 @@
         </is>
       </c>
       <c r="F675" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="676">
@@ -19793,7 +19793,7 @@
         </is>
       </c>
       <c r="F692" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="693">
@@ -19821,7 +19821,7 @@
         </is>
       </c>
       <c r="F693" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="694">
@@ -19849,7 +19849,7 @@
         </is>
       </c>
       <c r="F694" t="n">
-        <v>9</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="695">
@@ -19877,7 +19877,7 @@
         </is>
       </c>
       <c r="F695" t="n">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="696">
@@ -19905,7 +19905,7 @@
         </is>
       </c>
       <c r="F696" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="697">
@@ -19933,7 +19933,7 @@
         </is>
       </c>
       <c r="F697" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="698">
@@ -20017,7 +20017,7 @@
         </is>
       </c>
       <c r="F700" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="701">
@@ -20297,7 +20297,7 @@
         </is>
       </c>
       <c r="F710" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="711">
@@ -20465,7 +20465,7 @@
         </is>
       </c>
       <c r="F716" t="n">
-        <v>-1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="717">
@@ -20493,7 +20493,7 @@
         </is>
       </c>
       <c r="F717" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="718">
@@ -20717,7 +20717,7 @@
         </is>
       </c>
       <c r="F725" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="726">
@@ -20885,7 +20885,7 @@
         </is>
       </c>
       <c r="F731" t="n">
-        <v>9</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="732">
@@ -21025,7 +21025,7 @@
         </is>
       </c>
       <c r="F736" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="737">
@@ -21081,7 +21081,7 @@
         </is>
       </c>
       <c r="F738" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="739">
@@ -21193,7 +21193,7 @@
         </is>
       </c>
       <c r="F742" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="743">
@@ -21249,7 +21249,7 @@
         </is>
       </c>
       <c r="F744" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="745">
@@ -21277,7 +21277,7 @@
         </is>
       </c>
       <c r="F745" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="746">
@@ -21333,7 +21333,7 @@
         </is>
       </c>
       <c r="F747" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="748">
@@ -21529,7 +21529,7 @@
         </is>
       </c>
       <c r="F754" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="755">
@@ -21781,7 +21781,7 @@
         </is>
       </c>
       <c r="F763" t="n">
-        <v>-1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="764">
@@ -22089,7 +22089,7 @@
         </is>
       </c>
       <c r="F774" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="775">
@@ -22117,7 +22117,7 @@
         </is>
       </c>
       <c r="F775" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="776">
@@ -22565,7 +22565,7 @@
         </is>
       </c>
       <c r="F791" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="792">
@@ -22649,7 +22649,7 @@
         </is>
       </c>
       <c r="F794" t="n">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="795">
@@ -22733,7 +22733,7 @@
         </is>
       </c>
       <c r="F797" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="798">
@@ -22817,7 +22817,7 @@
         </is>
       </c>
       <c r="F800" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="801">
@@ -23041,7 +23041,7 @@
         </is>
       </c>
       <c r="F808" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="809">
@@ -23097,7 +23097,7 @@
         </is>
       </c>
       <c r="F810" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="811">
@@ -23237,7 +23237,7 @@
         </is>
       </c>
       <c r="F815" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="816">
@@ -23601,7 +23601,7 @@
         </is>
       </c>
       <c r="F828" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="829">
@@ -23769,7 +23769,7 @@
         </is>
       </c>
       <c r="F834" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="835">
@@ -23853,7 +23853,7 @@
         </is>
       </c>
       <c r="F837" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="838">
@@ -23881,7 +23881,7 @@
         </is>
       </c>
       <c r="F838" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="839">
@@ -23965,7 +23965,7 @@
         </is>
       </c>
       <c r="F841" t="n">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="842">
@@ -24021,7 +24021,7 @@
         </is>
       </c>
       <c r="F843" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="844">
@@ -24273,7 +24273,7 @@
         </is>
       </c>
       <c r="F852" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="853">
@@ -24469,7 +24469,7 @@
         </is>
       </c>
       <c r="F859" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="860">
@@ -24497,7 +24497,7 @@
         </is>
       </c>
       <c r="F860" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="861">
@@ -24525,7 +24525,7 @@
         </is>
       </c>
       <c r="F861" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="862">
@@ -24609,7 +24609,7 @@
         </is>
       </c>
       <c r="F864" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="865">
@@ -24721,7 +24721,7 @@
         </is>
       </c>
       <c r="F868" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="869">
@@ -24749,7 +24749,7 @@
         </is>
       </c>
       <c r="F869" t="n">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="870">
@@ -24889,7 +24889,7 @@
         </is>
       </c>
       <c r="F874" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="875">
@@ -25085,7 +25085,7 @@
         </is>
       </c>
       <c r="F881" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="882">
@@ -25113,7 +25113,7 @@
         </is>
       </c>
       <c r="F882" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="883">
@@ -25141,7 +25141,7 @@
         </is>
       </c>
       <c r="F883" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="884">
@@ -25449,7 +25449,7 @@
         </is>
       </c>
       <c r="F894" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="895">
@@ -25505,7 +25505,7 @@
         </is>
       </c>
       <c r="F896" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="897">
@@ -25701,7 +25701,7 @@
         </is>
       </c>
       <c r="F903" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="904">
@@ -25897,7 +25897,7 @@
         </is>
       </c>
       <c r="F910" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="911">
@@ -26037,7 +26037,7 @@
         </is>
       </c>
       <c r="F915" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="916">
@@ -26205,7 +26205,7 @@
         </is>
       </c>
       <c r="F921" t="n">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="922">
@@ -26429,7 +26429,7 @@
         </is>
       </c>
       <c r="F929" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="930">
@@ -26653,7 +26653,7 @@
         </is>
       </c>
       <c r="F937" t="n">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="938">
@@ -26821,7 +26821,7 @@
         </is>
       </c>
       <c r="F943" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="944">
@@ -26877,7 +26877,7 @@
         </is>
       </c>
       <c r="F945" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="946">
@@ -26961,7 +26961,7 @@
         </is>
       </c>
       <c r="F948" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="949">
@@ -27241,7 +27241,7 @@
         </is>
       </c>
       <c r="F958" t="n">
-        <v>8</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="959">
@@ -27689,7 +27689,7 @@
         </is>
       </c>
       <c r="F974" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="975">
@@ -27857,7 +27857,7 @@
         </is>
       </c>
       <c r="F980" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="981">
@@ -27913,7 +27913,7 @@
         </is>
       </c>
       <c r="F982" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="983">
@@ -27941,7 +27941,7 @@
         </is>
       </c>
       <c r="F983" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="984">
@@ -28277,7 +28277,7 @@
         </is>
       </c>
       <c r="F995" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="996">
@@ -28305,7 +28305,7 @@
         </is>
       </c>
       <c r="F996" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="997">
@@ -28333,7 +28333,7 @@
         </is>
       </c>
       <c r="F997" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="998">

</xml_diff>

<commit_message>
fix: update notebook indosbert and result
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>-1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>-1</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>4</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="12">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>9</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="14">
@@ -921,7 +921,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>-1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19">
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>-1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20">
@@ -1089,7 +1089,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>9</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="25">
@@ -1145,7 +1145,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="30">
@@ -1313,7 +1313,7 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33">
@@ -1341,7 +1341,7 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>7</v>
+        <v>27</v>
       </c>
     </row>
     <row r="34">
@@ -1369,7 +1369,7 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="35">
@@ -1509,7 +1509,7 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>-1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="40">
@@ -1649,7 +1649,7 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="45">
@@ -1677,7 +1677,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>6</v>
+        <v>37</v>
       </c>
     </row>
     <row r="46">
@@ -1705,7 +1705,7 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="47">
@@ -1845,7 +1845,7 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="52">
@@ -1901,7 +1901,7 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="54">
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>9</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="56">
@@ -2097,7 +2097,7 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>4</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="61">
@@ -2125,7 +2125,7 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>6</v>
+        <v>37</v>
       </c>
     </row>
     <row r="62">
@@ -2153,7 +2153,7 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="63">
@@ -2181,7 +2181,7 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>-1</v>
+        <v>40</v>
       </c>
     </row>
     <row r="64">
@@ -2293,7 +2293,7 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>-1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="68">
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="71">
@@ -2433,7 +2433,7 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="73">
@@ -2461,7 +2461,7 @@
         </is>
       </c>
       <c r="F73" t="n">
-        <v>-1</v>
+        <v>38</v>
       </c>
     </row>
     <row r="74">
@@ -2545,7 +2545,7 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>8</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="77">
@@ -2741,7 +2741,7 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>9</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="84">
@@ -2797,7 +2797,7 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="86">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>6</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="89">
@@ -2909,7 +2909,7 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>-1</v>
+        <v>39</v>
       </c>
     </row>
     <row r="90">
@@ -3133,7 +3133,7 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>6</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="98">
@@ -3217,7 +3217,7 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="101">
@@ -3273,7 +3273,7 @@
         </is>
       </c>
       <c r="F102" t="n">
-        <v>6</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="103">
@@ -3301,7 +3301,7 @@
         </is>
       </c>
       <c r="F103" t="n">
-        <v>-1</v>
+        <v>40</v>
       </c>
     </row>
     <row r="104">
@@ -3357,7 +3357,7 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>5</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="106">
@@ -3413,7 +3413,7 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>-1</v>
+        <v>28</v>
       </c>
     </row>
     <row r="108">
@@ -3441,7 +3441,7 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="109">
@@ -3469,7 +3469,7 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>-1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="110">
@@ -3497,7 +3497,7 @@
         </is>
       </c>
       <c r="F110" t="n">
-        <v>6</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="111">
@@ -3525,7 +3525,7 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="112">
@@ -3581,7 +3581,7 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="114">
@@ -3637,7 +3637,7 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="116">
@@ -3693,7 +3693,7 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="118">
@@ -3861,7 +3861,7 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="124">
@@ -3889,7 +3889,7 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>-1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="125">
@@ -4225,7 +4225,7 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="137">
@@ -4253,7 +4253,7 @@
         </is>
       </c>
       <c r="F137" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="138">
@@ -4785,7 +4785,7 @@
         </is>
       </c>
       <c r="F156" t="n">
-        <v>4</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="157">
@@ -5037,7 +5037,7 @@
         </is>
       </c>
       <c r="F165" t="n">
-        <v>-1</v>
+        <v>32</v>
       </c>
     </row>
     <row r="166">
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="F166" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
     </row>
     <row r="167">
@@ -5121,7 +5121,7 @@
         </is>
       </c>
       <c r="F168" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="169">
@@ -5205,7 +5205,7 @@
         </is>
       </c>
       <c r="F171" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="172">
@@ -5233,7 +5233,7 @@
         </is>
       </c>
       <c r="F172" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="173">
@@ -5317,7 +5317,7 @@
         </is>
       </c>
       <c r="F175" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="176">
@@ -5569,7 +5569,7 @@
         </is>
       </c>
       <c r="F184" t="n">
-        <v>-1</v>
+        <v>32</v>
       </c>
     </row>
     <row r="185">
@@ -5597,7 +5597,7 @@
         </is>
       </c>
       <c r="F185" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="186">
@@ -5681,7 +5681,7 @@
         </is>
       </c>
       <c r="F188" t="n">
-        <v>-1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="189">
@@ -5709,7 +5709,7 @@
         </is>
       </c>
       <c r="F189" t="n">
-        <v>-1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="190">
@@ -5765,7 +5765,7 @@
         </is>
       </c>
       <c r="F191" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="192">
@@ -5793,7 +5793,7 @@
         </is>
       </c>
       <c r="F192" t="n">
-        <v>-1</v>
+        <v>25</v>
       </c>
     </row>
     <row r="193">
@@ -5905,7 +5905,7 @@
         </is>
       </c>
       <c r="F196" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="197">
@@ -6017,7 +6017,7 @@
         </is>
       </c>
       <c r="F200" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="201">
@@ -6129,7 +6129,7 @@
         </is>
       </c>
       <c r="F204" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="205">
@@ -6185,7 +6185,7 @@
         </is>
       </c>
       <c r="F206" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="207">
@@ -6437,7 +6437,7 @@
         </is>
       </c>
       <c r="F215" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="216">
@@ -6577,7 +6577,7 @@
         </is>
       </c>
       <c r="F220" t="n">
-        <v>9</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="221">
@@ -6605,7 +6605,7 @@
         </is>
       </c>
       <c r="F221" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="222">
@@ -6661,7 +6661,7 @@
         </is>
       </c>
       <c r="F223" t="n">
-        <v>-1</v>
+        <v>28</v>
       </c>
     </row>
     <row r="224">
@@ -6689,7 +6689,7 @@
         </is>
       </c>
       <c r="F224" t="n">
-        <v>-1</v>
+        <v>39</v>
       </c>
     </row>
     <row r="225">
@@ -7025,7 +7025,7 @@
         </is>
       </c>
       <c r="F236" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="237">
@@ -7137,7 +7137,7 @@
         </is>
       </c>
       <c r="F240" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="241">
@@ -7165,7 +7165,7 @@
         </is>
       </c>
       <c r="F241" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="242">
@@ -7333,7 +7333,7 @@
         </is>
       </c>
       <c r="F247" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="248">
@@ -7417,7 +7417,7 @@
         </is>
       </c>
       <c r="F250" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="251">
@@ -7837,7 +7837,7 @@
         </is>
       </c>
       <c r="F265" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="266">
@@ -7865,7 +7865,7 @@
         </is>
       </c>
       <c r="F266" t="n">
-        <v>-1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="267">
@@ -7921,7 +7921,7 @@
         </is>
       </c>
       <c r="F268" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="269">
@@ -8061,7 +8061,7 @@
         </is>
       </c>
       <c r="F273" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="274">
@@ -8285,7 +8285,7 @@
         </is>
       </c>
       <c r="F281" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="282">
@@ -8565,7 +8565,7 @@
         </is>
       </c>
       <c r="F291" t="n">
-        <v>6</v>
+        <v>29</v>
       </c>
     </row>
     <row r="292">
@@ -8649,7 +8649,7 @@
         </is>
       </c>
       <c r="F294" t="n">
-        <v>-1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="295">
@@ -8761,7 +8761,7 @@
         </is>
       </c>
       <c r="F298" t="n">
-        <v>6</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="299">
@@ -8789,7 +8789,7 @@
         </is>
       </c>
       <c r="F299" t="n">
-        <v>-1</v>
+        <v>19</v>
       </c>
     </row>
     <row r="300">
@@ -8873,7 +8873,7 @@
         </is>
       </c>
       <c r="F302" t="n">
-        <v>-1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="303">
@@ -8901,7 +8901,7 @@
         </is>
       </c>
       <c r="F303" t="n">
-        <v>-1</v>
+        <v>33</v>
       </c>
     </row>
     <row r="304">
@@ -8985,7 +8985,7 @@
         </is>
       </c>
       <c r="F306" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="307">
@@ -9069,7 +9069,7 @@
         </is>
       </c>
       <c r="F309" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="310">
@@ -9405,7 +9405,7 @@
         </is>
       </c>
       <c r="F321" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="322">
@@ -9461,7 +9461,7 @@
         </is>
       </c>
       <c r="F323" t="n">
-        <v>-1</v>
+        <v>31</v>
       </c>
     </row>
     <row r="324">
@@ -9601,7 +9601,7 @@
         </is>
       </c>
       <c r="F328" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="329">
@@ -9713,7 +9713,7 @@
         </is>
       </c>
       <c r="F332" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="333">
@@ -9797,7 +9797,7 @@
         </is>
       </c>
       <c r="F335" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="336">
@@ -9909,7 +9909,7 @@
         </is>
       </c>
       <c r="F339" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="340">
@@ -9993,7 +9993,7 @@
         </is>
       </c>
       <c r="F342" t="n">
-        <v>-1</v>
+        <v>40</v>
       </c>
     </row>
     <row r="343">
@@ -10077,7 +10077,7 @@
         </is>
       </c>
       <c r="F345" t="n">
-        <v>6</v>
+        <v>37</v>
       </c>
     </row>
     <row r="346">
@@ -10189,7 +10189,7 @@
         </is>
       </c>
       <c r="F349" t="n">
-        <v>9</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="350">
@@ -10217,7 +10217,7 @@
         </is>
       </c>
       <c r="F350" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="351">
@@ -10357,7 +10357,7 @@
         </is>
       </c>
       <c r="F355" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="356">
@@ -10385,7 +10385,7 @@
         </is>
       </c>
       <c r="F356" t="n">
-        <v>-1</v>
+        <v>40</v>
       </c>
     </row>
     <row r="357">
@@ -10525,7 +10525,7 @@
         </is>
       </c>
       <c r="F361" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="362">
@@ -10581,7 +10581,7 @@
         </is>
       </c>
       <c r="F363" t="n">
-        <v>-1</v>
+        <v>19</v>
       </c>
     </row>
     <row r="364">
@@ -10693,7 +10693,7 @@
         </is>
       </c>
       <c r="F367" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="368">
@@ -10805,7 +10805,7 @@
         </is>
       </c>
       <c r="F371" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="372">
@@ -10861,7 +10861,7 @@
         </is>
       </c>
       <c r="F373" t="n">
-        <v>-1</v>
+        <v>21</v>
       </c>
     </row>
     <row r="374">
@@ -10945,7 +10945,7 @@
         </is>
       </c>
       <c r="F376" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="377">
@@ -11113,7 +11113,7 @@
         </is>
       </c>
       <c r="F382" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="383">
@@ -11141,7 +11141,7 @@
         </is>
       </c>
       <c r="F383" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="384">
@@ -11225,7 +11225,7 @@
         </is>
       </c>
       <c r="F386" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="387">
@@ -11253,7 +11253,7 @@
         </is>
       </c>
       <c r="F387" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="388">
@@ -11505,7 +11505,7 @@
         </is>
       </c>
       <c r="F396" t="n">
-        <v>7</v>
+        <v>27</v>
       </c>
     </row>
     <row r="397">
@@ -11533,7 +11533,7 @@
         </is>
       </c>
       <c r="F397" t="n">
-        <v>-1</v>
+        <v>32</v>
       </c>
     </row>
     <row r="398">
@@ -11645,7 +11645,7 @@
         </is>
       </c>
       <c r="F401" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="402">
@@ -11701,7 +11701,7 @@
         </is>
       </c>
       <c r="F403" t="n">
-        <v>-1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="404">
@@ -11729,7 +11729,7 @@
         </is>
       </c>
       <c r="F404" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="405">
@@ -11897,7 +11897,7 @@
         </is>
       </c>
       <c r="F410" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="411">
@@ -11925,7 +11925,7 @@
         </is>
       </c>
       <c r="F411" t="n">
-        <v>-1</v>
+        <v>28</v>
       </c>
     </row>
     <row r="412">
@@ -11953,7 +11953,7 @@
         </is>
       </c>
       <c r="F412" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="413">
@@ -12149,7 +12149,7 @@
         </is>
       </c>
       <c r="F419" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="420">
@@ -12345,7 +12345,7 @@
         </is>
       </c>
       <c r="F426" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="427">
@@ -12429,7 +12429,7 @@
         </is>
       </c>
       <c r="F429" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="430">
@@ -12457,7 +12457,7 @@
         </is>
       </c>
       <c r="F430" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="431">
@@ -12681,7 +12681,7 @@
         </is>
       </c>
       <c r="F438" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="439">
@@ -12709,7 +12709,7 @@
         </is>
       </c>
       <c r="F439" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="440">
@@ -12765,7 +12765,7 @@
         </is>
       </c>
       <c r="F441" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="442">
@@ -12793,7 +12793,7 @@
         </is>
       </c>
       <c r="F442" t="n">
-        <v>9</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="443">
@@ -12961,7 +12961,7 @@
         </is>
       </c>
       <c r="F448" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="449">
@@ -13045,7 +13045,7 @@
         </is>
       </c>
       <c r="F451" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="452">
@@ -13129,7 +13129,7 @@
         </is>
       </c>
       <c r="F454" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="455">
@@ -13241,7 +13241,7 @@
         </is>
       </c>
       <c r="F458" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="459">
@@ -13269,7 +13269,7 @@
         </is>
       </c>
       <c r="F459" t="n">
-        <v>-1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="460">
@@ -13297,7 +13297,7 @@
         </is>
       </c>
       <c r="F460" t="n">
-        <v>6</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="461">
@@ -13437,7 +13437,7 @@
         </is>
       </c>
       <c r="F465" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="466">
@@ -13465,7 +13465,7 @@
         </is>
       </c>
       <c r="F466" t="n">
-        <v>-1</v>
+        <v>22</v>
       </c>
     </row>
     <row r="467">
@@ -13633,7 +13633,7 @@
         </is>
       </c>
       <c r="F472" t="n">
-        <v>-1</v>
+        <v>21</v>
       </c>
     </row>
     <row r="473">
@@ -13689,7 +13689,7 @@
         </is>
       </c>
       <c r="F474" t="n">
-        <v>-1</v>
+        <v>38</v>
       </c>
     </row>
     <row r="475">
@@ -13773,7 +13773,7 @@
         </is>
       </c>
       <c r="F477" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="478">
@@ -13801,7 +13801,7 @@
         </is>
       </c>
       <c r="F478" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="479">
@@ -13913,7 +13913,7 @@
         </is>
       </c>
       <c r="F482" t="n">
-        <v>-1</v>
+        <v>21</v>
       </c>
     </row>
     <row r="483">
@@ -14053,7 +14053,7 @@
         </is>
       </c>
       <c r="F487" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="488">
@@ -14081,7 +14081,7 @@
         </is>
       </c>
       <c r="F488" t="n">
-        <v>6</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="489">
@@ -14193,7 +14193,7 @@
         </is>
       </c>
       <c r="F492" t="n">
-        <v>9</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="493">
@@ -14249,7 +14249,7 @@
         </is>
       </c>
       <c r="F494" t="n">
-        <v>-1</v>
+        <v>22</v>
       </c>
     </row>
     <row r="495">
@@ -14417,7 +14417,7 @@
         </is>
       </c>
       <c r="F500" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="501">
@@ -14557,7 +14557,7 @@
         </is>
       </c>
       <c r="F505" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="506">
@@ -14781,7 +14781,7 @@
         </is>
       </c>
       <c r="F513" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
     </row>
     <row r="514">
@@ -14977,7 +14977,7 @@
         </is>
       </c>
       <c r="F520" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="521">
@@ -15061,7 +15061,7 @@
         </is>
       </c>
       <c r="F523" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="524">
@@ -15117,7 +15117,7 @@
         </is>
       </c>
       <c r="F525" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
     </row>
     <row r="526">
@@ -15257,7 +15257,7 @@
         </is>
       </c>
       <c r="F530" t="n">
-        <v>-1</v>
+        <v>33</v>
       </c>
     </row>
     <row r="531">
@@ -15341,7 +15341,7 @@
         </is>
       </c>
       <c r="F533" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="534">
@@ -15453,7 +15453,7 @@
         </is>
       </c>
       <c r="F537" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="538">
@@ -15509,7 +15509,7 @@
         </is>
       </c>
       <c r="F539" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="540">
@@ -15537,7 +15537,7 @@
         </is>
       </c>
       <c r="F540" t="n">
-        <v>-1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="541">
@@ -15565,7 +15565,7 @@
         </is>
       </c>
       <c r="F541" t="n">
-        <v>6</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="542">
@@ -15621,7 +15621,7 @@
         </is>
       </c>
       <c r="F543" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="544">
@@ -15873,7 +15873,7 @@
         </is>
       </c>
       <c r="F552" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="553">
@@ -15929,7 +15929,7 @@
         </is>
       </c>
       <c r="F554" t="n">
-        <v>-1</v>
+        <v>24</v>
       </c>
     </row>
     <row r="555">
@@ -16097,7 +16097,7 @@
         </is>
       </c>
       <c r="F560" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="561">
@@ -16125,7 +16125,7 @@
         </is>
       </c>
       <c r="F561" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="562">
@@ -16265,7 +16265,7 @@
         </is>
       </c>
       <c r="F566" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="567">
@@ -16293,7 +16293,7 @@
         </is>
       </c>
       <c r="F567" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="568">
@@ -16349,7 +16349,7 @@
         </is>
       </c>
       <c r="F569" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
     </row>
     <row r="570">
@@ -16377,7 +16377,7 @@
         </is>
       </c>
       <c r="F570" t="n">
-        <v>-1</v>
+        <v>34</v>
       </c>
     </row>
     <row r="571">
@@ -16489,7 +16489,7 @@
         </is>
       </c>
       <c r="F574" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="575">
@@ -16517,7 +16517,7 @@
         </is>
       </c>
       <c r="F575" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
     </row>
     <row r="576">
@@ -16545,7 +16545,7 @@
         </is>
       </c>
       <c r="F576" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="577">
@@ -16685,7 +16685,7 @@
         </is>
       </c>
       <c r="F581" t="n">
-        <v>-1</v>
+        <v>33</v>
       </c>
     </row>
     <row r="582">
@@ -16741,7 +16741,7 @@
         </is>
       </c>
       <c r="F583" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="584">
@@ -17077,7 +17077,7 @@
         </is>
       </c>
       <c r="F595" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="596">
@@ -17161,7 +17161,7 @@
         </is>
       </c>
       <c r="F598" t="n">
-        <v>-1</v>
+        <v>34</v>
       </c>
     </row>
     <row r="599">
@@ -17329,7 +17329,7 @@
         </is>
       </c>
       <c r="F604" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
     </row>
     <row r="605">
@@ -17469,7 +17469,7 @@
         </is>
       </c>
       <c r="F609" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="610">
@@ -17525,7 +17525,7 @@
         </is>
       </c>
       <c r="F611" t="n">
-        <v>-1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="612">
@@ -17581,7 +17581,7 @@
         </is>
       </c>
       <c r="F613" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="614">
@@ -17609,7 +17609,7 @@
         </is>
       </c>
       <c r="F614" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="615">
@@ -17665,7 +17665,7 @@
         </is>
       </c>
       <c r="F616" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="617">
@@ -17693,7 +17693,7 @@
         </is>
       </c>
       <c r="F617" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="618">
@@ -17917,7 +17917,7 @@
         </is>
       </c>
       <c r="F625" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="626">
@@ -18001,7 +18001,7 @@
         </is>
       </c>
       <c r="F628" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="629">
@@ -18057,7 +18057,7 @@
         </is>
       </c>
       <c r="F630" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="631">
@@ -18141,7 +18141,7 @@
         </is>
       </c>
       <c r="F633" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="634">
@@ -18169,7 +18169,7 @@
         </is>
       </c>
       <c r="F634" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
     </row>
     <row r="635">
@@ -18225,7 +18225,7 @@
         </is>
       </c>
       <c r="F636" t="n">
-        <v>9</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="637">
@@ -18393,7 +18393,7 @@
         </is>
       </c>
       <c r="F642" t="n">
-        <v>-1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="643">
@@ -18449,7 +18449,7 @@
         </is>
       </c>
       <c r="F644" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="645">
@@ -18477,7 +18477,7 @@
         </is>
       </c>
       <c r="F645" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="646">
@@ -18505,7 +18505,7 @@
         </is>
       </c>
       <c r="F646" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="647">
@@ -18533,7 +18533,7 @@
         </is>
       </c>
       <c r="F647" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="648">
@@ -18589,7 +18589,7 @@
         </is>
       </c>
       <c r="F649" t="n">
-        <v>9</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="650">
@@ -18617,7 +18617,7 @@
         </is>
       </c>
       <c r="F650" t="n">
-        <v>-1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="651">
@@ -18701,7 +18701,7 @@
         </is>
       </c>
       <c r="F653" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="654">
@@ -18757,7 +18757,7 @@
         </is>
       </c>
       <c r="F655" t="n">
-        <v>-1</v>
+        <v>39</v>
       </c>
     </row>
     <row r="656">
@@ -18841,7 +18841,7 @@
         </is>
       </c>
       <c r="F658" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="659">
@@ -18925,7 +18925,7 @@
         </is>
       </c>
       <c r="F661" t="n">
-        <v>-1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="662">
@@ -19121,7 +19121,7 @@
         </is>
       </c>
       <c r="F668" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
     </row>
     <row r="669">
@@ -19149,7 +19149,7 @@
         </is>
       </c>
       <c r="F669" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="670">
@@ -19177,7 +19177,7 @@
         </is>
       </c>
       <c r="F670" t="n">
-        <v>7</v>
+        <v>36</v>
       </c>
     </row>
     <row r="671">
@@ -19289,7 +19289,7 @@
         </is>
       </c>
       <c r="F674" t="n">
-        <v>10</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="675">
@@ -19317,7 +19317,7 @@
         </is>
       </c>
       <c r="F675" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="676">
@@ -19793,7 +19793,7 @@
         </is>
       </c>
       <c r="F692" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="693">
@@ -19821,7 +19821,7 @@
         </is>
       </c>
       <c r="F693" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="694">
@@ -19849,7 +19849,7 @@
         </is>
       </c>
       <c r="F694" t="n">
-        <v>-1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="695">
@@ -19877,7 +19877,7 @@
         </is>
       </c>
       <c r="F695" t="n">
-        <v>10</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="696">
@@ -19905,7 +19905,7 @@
         </is>
       </c>
       <c r="F696" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="697">
@@ -19933,7 +19933,7 @@
         </is>
       </c>
       <c r="F697" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="698">
@@ -20129,7 +20129,7 @@
         </is>
       </c>
       <c r="F704" t="n">
-        <v>-1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="705">
@@ -20213,7 +20213,7 @@
         </is>
       </c>
       <c r="F707" t="n">
-        <v>-1</v>
+        <v>19</v>
       </c>
     </row>
     <row r="708">
@@ -20297,7 +20297,7 @@
         </is>
       </c>
       <c r="F710" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="711">
@@ -20465,7 +20465,7 @@
         </is>
       </c>
       <c r="F716" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="717">
@@ -20493,7 +20493,7 @@
         </is>
       </c>
       <c r="F717" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="718">
@@ -20605,7 +20605,7 @@
         </is>
       </c>
       <c r="F721" t="n">
-        <v>-1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="722">
@@ -20717,7 +20717,7 @@
         </is>
       </c>
       <c r="F725" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="726">
@@ -20745,7 +20745,7 @@
         </is>
       </c>
       <c r="F726" t="n">
-        <v>-1</v>
+        <v>24</v>
       </c>
     </row>
     <row r="727">
@@ -20885,7 +20885,7 @@
         </is>
       </c>
       <c r="F731" t="n">
-        <v>-1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="732">
@@ -21025,7 +21025,7 @@
         </is>
       </c>
       <c r="F736" t="n">
-        <v>6</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="737">
@@ -21081,7 +21081,7 @@
         </is>
       </c>
       <c r="F738" t="n">
-        <v>4</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="739">
@@ -21193,7 +21193,7 @@
         </is>
       </c>
       <c r="F742" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="743">
@@ -21249,7 +21249,7 @@
         </is>
       </c>
       <c r="F744" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="745">
@@ -21277,7 +21277,7 @@
         </is>
       </c>
       <c r="F745" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="746">
@@ -21333,7 +21333,7 @@
         </is>
       </c>
       <c r="F747" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="748">
@@ -21417,7 +21417,7 @@
         </is>
       </c>
       <c r="F750" t="n">
-        <v>-1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="751">
@@ -21529,7 +21529,7 @@
         </is>
       </c>
       <c r="F754" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="755">
@@ -21781,7 +21781,7 @@
         </is>
       </c>
       <c r="F763" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="764">
@@ -22089,7 +22089,7 @@
         </is>
       </c>
       <c r="F774" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="775">
@@ -22117,7 +22117,7 @@
         </is>
       </c>
       <c r="F775" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="776">
@@ -22285,7 +22285,7 @@
         </is>
       </c>
       <c r="F781" t="n">
-        <v>-1</v>
+        <v>31</v>
       </c>
     </row>
     <row r="782">
@@ -22313,7 +22313,7 @@
         </is>
       </c>
       <c r="F782" t="n">
-        <v>-1</v>
+        <v>31</v>
       </c>
     </row>
     <row r="783">
@@ -22537,7 +22537,7 @@
         </is>
       </c>
       <c r="F790" t="n">
-        <v>-1</v>
+        <v>22</v>
       </c>
     </row>
     <row r="791">
@@ -22565,7 +22565,7 @@
         </is>
       </c>
       <c r="F791" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="792">
@@ -22649,7 +22649,7 @@
         </is>
       </c>
       <c r="F794" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="795">
@@ -22733,7 +22733,7 @@
         </is>
       </c>
       <c r="F797" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="798">
@@ -22817,7 +22817,7 @@
         </is>
       </c>
       <c r="F800" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
     </row>
     <row r="801">
@@ -22845,7 +22845,7 @@
         </is>
       </c>
       <c r="F801" t="n">
-        <v>-1</v>
+        <v>24</v>
       </c>
     </row>
     <row r="802">
@@ -23041,7 +23041,7 @@
         </is>
       </c>
       <c r="F808" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="809">
@@ -23097,7 +23097,7 @@
         </is>
       </c>
       <c r="F810" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="811">
@@ -23237,7 +23237,7 @@
         </is>
       </c>
       <c r="F815" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="816">
@@ -23601,7 +23601,7 @@
         </is>
       </c>
       <c r="F828" t="n">
-        <v>4</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="829">
@@ -23769,7 +23769,7 @@
         </is>
       </c>
       <c r="F834" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="835">
@@ -23797,7 +23797,7 @@
         </is>
       </c>
       <c r="F835" t="n">
-        <v>-1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="836">
@@ -23853,7 +23853,7 @@
         </is>
       </c>
       <c r="F837" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="838">
@@ -23881,7 +23881,7 @@
         </is>
       </c>
       <c r="F838" t="n">
-        <v>7</v>
+        <v>36</v>
       </c>
     </row>
     <row r="839">
@@ -23965,7 +23965,7 @@
         </is>
       </c>
       <c r="F841" t="n">
-        <v>10</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="842">
@@ -24021,7 +24021,7 @@
         </is>
       </c>
       <c r="F843" t="n">
-        <v>7</v>
+        <v>27</v>
       </c>
     </row>
     <row r="844">
@@ -24273,7 +24273,7 @@
         </is>
       </c>
       <c r="F852" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="853">
@@ -24385,7 +24385,7 @@
         </is>
       </c>
       <c r="F856" t="n">
-        <v>-1</v>
+        <v>36</v>
       </c>
     </row>
     <row r="857">
@@ -24469,7 +24469,7 @@
         </is>
       </c>
       <c r="F859" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="860">
@@ -24497,7 +24497,7 @@
         </is>
       </c>
       <c r="F860" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="861">
@@ -24525,7 +24525,7 @@
         </is>
       </c>
       <c r="F861" t="n">
-        <v>7</v>
+        <v>27</v>
       </c>
     </row>
     <row r="862">
@@ -24609,7 +24609,7 @@
         </is>
       </c>
       <c r="F864" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="865">
@@ -24721,7 +24721,7 @@
         </is>
       </c>
       <c r="F868" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="869">
@@ -24749,7 +24749,7 @@
         </is>
       </c>
       <c r="F869" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="870">
@@ -24889,7 +24889,7 @@
         </is>
       </c>
       <c r="F874" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="875">
@@ -25057,7 +25057,7 @@
         </is>
       </c>
       <c r="F880" t="n">
-        <v>-1</v>
+        <v>22</v>
       </c>
     </row>
     <row r="881">
@@ -25085,7 +25085,7 @@
         </is>
       </c>
       <c r="F881" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="882">
@@ -25113,7 +25113,7 @@
         </is>
       </c>
       <c r="F882" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="883">
@@ -25141,7 +25141,7 @@
         </is>
       </c>
       <c r="F883" t="n">
-        <v>6</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="884">
@@ -25309,7 +25309,7 @@
         </is>
       </c>
       <c r="F889" t="n">
-        <v>-1</v>
+        <v>22</v>
       </c>
     </row>
     <row r="890">
@@ -25449,7 +25449,7 @@
         </is>
       </c>
       <c r="F894" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="895">
@@ -25505,7 +25505,7 @@
         </is>
       </c>
       <c r="F896" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="897">
@@ -25561,7 +25561,7 @@
         </is>
       </c>
       <c r="F898" t="n">
-        <v>-1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="899">
@@ -25701,7 +25701,7 @@
         </is>
       </c>
       <c r="F903" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="904">
@@ -25757,7 +25757,7 @@
         </is>
       </c>
       <c r="F905" t="n">
-        <v>-1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="906">
@@ -25785,7 +25785,7 @@
         </is>
       </c>
       <c r="F906" t="n">
-        <v>-1</v>
+        <v>25</v>
       </c>
     </row>
     <row r="907">
@@ -25897,7 +25897,7 @@
         </is>
       </c>
       <c r="F910" t="n">
-        <v>7</v>
+        <v>36</v>
       </c>
     </row>
     <row r="911">
@@ -26037,7 +26037,7 @@
         </is>
       </c>
       <c r="F915" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="916">
@@ -26205,7 +26205,7 @@
         </is>
       </c>
       <c r="F921" t="n">
-        <v>9</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="922">
@@ -26345,7 +26345,7 @@
         </is>
       </c>
       <c r="F926" t="n">
-        <v>-1</v>
+        <v>19</v>
       </c>
     </row>
     <row r="927">
@@ -26429,7 +26429,7 @@
         </is>
       </c>
       <c r="F929" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="930">
@@ -26597,7 +26597,7 @@
         </is>
       </c>
       <c r="F935" t="n">
-        <v>-1</v>
+        <v>22</v>
       </c>
     </row>
     <row r="936">
@@ -26653,7 +26653,7 @@
         </is>
       </c>
       <c r="F937" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="938">
@@ -26793,7 +26793,7 @@
         </is>
       </c>
       <c r="F942" t="n">
-        <v>-1</v>
+        <v>38</v>
       </c>
     </row>
     <row r="943">
@@ -26821,7 +26821,7 @@
         </is>
       </c>
       <c r="F943" t="n">
-        <v>4</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="944">
@@ -26877,7 +26877,7 @@
         </is>
       </c>
       <c r="F945" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="946">
@@ -26961,7 +26961,7 @@
         </is>
       </c>
       <c r="F948" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="949">
@@ -27213,7 +27213,7 @@
         </is>
       </c>
       <c r="F957" t="n">
-        <v>-1</v>
+        <v>22</v>
       </c>
     </row>
     <row r="958">
@@ -27241,7 +27241,7 @@
         </is>
       </c>
       <c r="F958" t="n">
-        <v>-1</v>
+        <v>21</v>
       </c>
     </row>
     <row r="959">
@@ -27297,7 +27297,7 @@
         </is>
       </c>
       <c r="F960" t="n">
-        <v>-1</v>
+        <v>34</v>
       </c>
     </row>
     <row r="961">
@@ -27689,7 +27689,7 @@
         </is>
       </c>
       <c r="F974" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="975">
@@ -27857,7 +27857,7 @@
         </is>
       </c>
       <c r="F980" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="981">
@@ -27913,7 +27913,7 @@
         </is>
       </c>
       <c r="F982" t="n">
-        <v>4</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="983">
@@ -27941,7 +27941,7 @@
         </is>
       </c>
       <c r="F983" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="984">
@@ -28277,7 +28277,7 @@
         </is>
       </c>
       <c r="F995" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="996">
@@ -28305,7 +28305,7 @@
         </is>
       </c>
       <c r="F996" t="n">
-        <v>6</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="997">
@@ -28333,7 +28333,7 @@
         </is>
       </c>
       <c r="F997" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="998">

</xml_diff>